<commit_message>
enhance weekly audit and sort data stock by type 3
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryuta\OneDrive\Documents\coding shit\Thanaka-Shop-Auditor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD621913-8340-435D-AC49-4CF878910607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56664C03-B6FD-4F40-BFA2-8D736DE3E3FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C17C1E5D-89FB-4119-AB7A-F64E2B3B0F2B}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
-  <si>
-    <t>สบู่ทานาคา</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
   <si>
     <t>1 ก้อน</t>
   </si>
@@ -59,12 +56,6 @@
     <t>Quantity sold</t>
   </si>
   <si>
-    <t>สบู่ทับทิม</t>
-  </si>
-  <si>
-    <t>ครีมซองทานาคา</t>
-  </si>
-  <si>
     <t>1 ซอง</t>
   </si>
   <si>
@@ -74,24 +65,12 @@
     <t>6 ซอง (1 กล่อง)</t>
   </si>
   <si>
-    <t>ครีมซองทับทิม</t>
-  </si>
-  <si>
-    <t>ครีมกระปุกทานาคา</t>
-  </si>
-  <si>
     <t>1 กล่อง 6 ซอง</t>
   </si>
   <si>
     <t>2 กล่อง 12 ซอง</t>
   </si>
   <si>
-    <t>ครีมกระปุกทับทิม</t>
-  </si>
-  <si>
-    <t>แป้งทานาคา 80 กรัม</t>
-  </si>
-  <si>
     <t>1 กระป๋อง</t>
   </si>
   <si>
@@ -101,21 +80,9 @@
     <t>6 กระป๋อง</t>
   </si>
   <si>
-    <t>แป้งทานาคา 180 กรัม</t>
-  </si>
-  <si>
-    <t>แป้งซาติน</t>
-  </si>
-  <si>
     <t>สบู่แพ็ค 3+3</t>
   </si>
   <si>
-    <t>สบู่เหลวทับทิม 1 ขวด</t>
-  </si>
-  <si>
-    <t>สบู่เหลวทานาคา 1 ขวด</t>
-  </si>
-  <si>
     <t>เซ็ตทดลองทับทิม (สบู่ + ครีม)</t>
   </si>
   <si>
@@ -123,13 +90,163 @@
   </si>
   <si>
     <t>เซ็ตสบู่ก้อน (ทานาคา + ทับทิม)</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>tan_soap</t>
+  </si>
+  <si>
+    <t>tan_soap_3</t>
+  </si>
+  <si>
+    <t>tan_soap_6</t>
+  </si>
+  <si>
+    <t>pom_soap</t>
+  </si>
+  <si>
+    <t>pom_soap_3</t>
+  </si>
+  <si>
+    <t>pom_soap_6</t>
+  </si>
+  <si>
+    <t>tan_lqd</t>
+  </si>
+  <si>
+    <t>pom_lqd</t>
+  </si>
+  <si>
+    <t>tan_cr_sch</t>
+  </si>
+  <si>
+    <t>tan_cr_sch_3</t>
+  </si>
+  <si>
+    <t>tan_cr_sch_6</t>
+  </si>
+  <si>
+    <t>tan_cr_sch_12</t>
+  </si>
+  <si>
+    <t>pom_cr_sch</t>
+  </si>
+  <si>
+    <t>pom_cr_sch_3</t>
+  </si>
+  <si>
+    <t>pom_cr_sch_6</t>
+  </si>
+  <si>
+    <t>tan_cr_jar</t>
+  </si>
+  <si>
+    <t>pom_cr_jar</t>
+  </si>
+  <si>
+    <t>powder_80</t>
+  </si>
+  <si>
+    <t>powder_80_3</t>
+  </si>
+  <si>
+    <t>powder_80_6</t>
+  </si>
+  <si>
+    <t>powder_180</t>
+  </si>
+  <si>
+    <t>satin</t>
+  </si>
+  <si>
+    <t>satin_3</t>
+  </si>
+  <si>
+    <t>satin_6</t>
+  </si>
+  <si>
+    <t>pom_test</t>
+  </si>
+  <si>
+    <t>tan_test</t>
+  </si>
+  <si>
+    <t>soap_bundle_1_1</t>
+  </si>
+  <si>
+    <t>soap_bundle_3_3</t>
+  </si>
+  <si>
+    <t>เซ็ตสบู่เหลว (ทานาคา + ทับทิม)</t>
+  </si>
+  <si>
+    <t>lqd_combo</t>
+  </si>
+  <si>
+    <t>เซ็ตครีมซอง (ทานาคา + ทับทิม)</t>
+  </si>
+  <si>
+    <t>sch_bundle</t>
+  </si>
+  <si>
+    <t>tan_lqd_2</t>
+  </si>
+  <si>
+    <t>pom_lqd_2</t>
+  </si>
+  <si>
+    <t>1 ขวด</t>
+  </si>
+  <si>
+    <t>2 ขวด</t>
+  </si>
+  <si>
+    <t>tan_soap_12</t>
+  </si>
+  <si>
+    <t>12 ก้อน</t>
+  </si>
+  <si>
+    <t>thanaka soap</t>
+  </si>
+  <si>
+    <t>promegranate soap</t>
+  </si>
+  <si>
+    <t>thanaka liquid soap</t>
+  </si>
+  <si>
+    <t>promegranate liquid soap</t>
+  </si>
+  <si>
+    <t>thanaka cream sachet</t>
+  </si>
+  <si>
+    <t>promegranate cream sachet</t>
+  </si>
+  <si>
+    <t>thanaka cream jar</t>
+  </si>
+  <si>
+    <t>promegranate cream jar</t>
+  </si>
+  <si>
+    <t>thanaka powder 80 g</t>
+  </si>
+  <si>
+    <t>thanaka powder 180 g</t>
+  </si>
+  <si>
+    <t>satin powder</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +259,13 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="ChulaCharasNew"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="222"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -506,184 +630,319 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15043B8A-F2E8-48EA-888B-AED9D7F6659E}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="20.69921875" defaultRowHeight="33.6" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.296875" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="20.69921875" style="2"/>
+    <col min="1" max="1" width="20.69921875" style="1"/>
+    <col min="2" max="2" width="26.296875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="20.69921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="14" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>27</v>
+    <row r="33" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="B1:C1"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>